<commit_message>
Update dashboard screenshot with real Excel view and clean currency format mask
</commit_message>
<xml_diff>
--- a/Stock_Portfolio_Master_Complete_v2.xlsx
+++ b/Stock_Portfolio_Master_Complete_v2.xlsx
@@ -50,55 +50,55 @@
     <t>SELECT STOCK TO ANALYZE:</t>
   </si>
   <si>
+    <t>TCS</t>
+  </si>
+  <si>
+    <t>HOLDING MARKET VALUE</t>
+  </si>
+  <si>
+    <t>TODAY'S GAIN / LOSS</t>
+  </si>
+  <si>
+    <t>TODAY'S CHANGE (%)</t>
+  </si>
+  <si>
+    <t>UNREALISED GAIN/(LOSS)</t>
+  </si>
+  <si>
+    <t>TOTAL RETURN (%)</t>
+  </si>
+  <si>
+    <t>Asset / Stock Name</t>
+  </si>
+  <si>
+    <t>Sector / Industry</t>
+  </si>
+  <si>
+    <t>Units (Shares)</t>
+  </si>
+  <si>
+    <t>Current Price (CMP)</t>
+  </si>
+  <si>
+    <t>Market Value</t>
+  </si>
+  <si>
+    <t>Today's Change</t>
+  </si>
+  <si>
+    <t>Today's %</t>
+  </si>
+  <si>
+    <t>Total Gain / Loss</t>
+  </si>
+  <si>
+    <t>12M Trend Graph</t>
+  </si>
+  <si>
     <t>HCL TECH</t>
   </si>
   <si>
-    <t>HOLDING MARKET VALUE</t>
-  </si>
-  <si>
-    <t>TODAY'S GAIN / LOSS</t>
-  </si>
-  <si>
-    <t>TODAY'S CHANGE (%)</t>
-  </si>
-  <si>
-    <t>UNREALISED GAIN/(LOSS)</t>
-  </si>
-  <si>
-    <t>TOTAL RETURN (%)</t>
-  </si>
-  <si>
-    <t>Asset / Stock Name</t>
-  </si>
-  <si>
-    <t>Sector / Industry</t>
-  </si>
-  <si>
-    <t>Units (Shares)</t>
-  </si>
-  <si>
-    <t>Current Price (CMP)</t>
-  </si>
-  <si>
-    <t>Market Value</t>
-  </si>
-  <si>
-    <t>Today's Change</t>
-  </si>
-  <si>
-    <t>Today's %</t>
-  </si>
-  <si>
-    <t>Total Gain / Loss</t>
-  </si>
-  <si>
-    <t>12M Trend Graph</t>
-  </si>
-  <si>
     <t>Information Technology</t>
-  </si>
-  <si>
-    <t>TCS</t>
   </si>
   <si>
     <t>INFOSYS</t>
@@ -637,7 +637,7 @@
     <numFmt numFmtId="164" formatCode="&quot;₹ &quot;#,##0.00"/>
     <numFmt numFmtId="165" formatCode="+0.00%;-0.00%;0.00%"/>
     <numFmt numFmtId="166" formatCode="#,##0"/>
-    <numFmt numFmtId="167" formatCode="&quot;+&quot;₹ &quot;#,##0.00;(&quot;-&quot;₹ &quot;#,##0.00);&quot;₹ &quot;0.00"/>
+    <numFmt numFmtId="167" formatCode="&quot;₹ &quot;#,##0.00;[Red](&quot;₹ &quot;#,##0.00);&quot;₹ &quot;0.00"/>
     <numFmt numFmtId="168" formatCode="0.00"/>
     <numFmt numFmtId="169" formatCode="@"/>
   </numFmts>
@@ -1125,14 +1125,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
-    <dxf>
-      <font>
-        <b/>
-        <color rgb="FFDC2626"/>
-      </font>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
 </styleSheet>
 </file>
@@ -3151,10 +3144,10 @@
     </row>
     <row r="6" spans="2:10" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="11" t="s">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D6" s="13">
         <v>150</v>
@@ -3179,10 +3172,10 @@
     </row>
     <row r="7" spans="2:10" ht="22" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="18" t="s">
+        <v>2</v>
+      </c>
+      <c r="C7" s="19" t="s">
         <v>18</v>
-      </c>
-      <c r="C7" s="19" t="s">
-        <v>17</v>
       </c>
       <c r="D7" s="20">
         <v>40</v>
@@ -3210,7 +3203,7 @@
         <v>19</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D8" s="13">
         <v>120</v>
@@ -3238,7 +3231,7 @@
         <v>20</v>
       </c>
       <c r="C9" s="19" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D9" s="20">
         <v>250</v>
@@ -3266,7 +3259,7 @@
         <v>21</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D10" s="13">
         <v>80</v>
@@ -3726,11 +3719,6 @@
           <x14:id>{DA7ABA51-AAAA-BBBB-0001-000000000001}</x14:id>
         </ext>
       </extLst>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I6:I16">
-    <cfRule type="cellIs" dxfId="0" priority="2" operator="lessThan">
-      <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
@@ -4028,13 +4016,13 @@
         <v>68</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="C2" s="12" t="s">
         <v>69</v>
       </c>
       <c r="D2" s="12" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E2" s="13">
         <v>150</v>
@@ -4089,13 +4077,13 @@
         <v>73</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="C3" s="12" t="s">
         <v>74</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E3" s="13">
         <v>40</v>
@@ -4156,7 +4144,7 @@
         <v>79</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E4" s="13">
         <v>120</v>
@@ -4217,7 +4205,7 @@
         <v>84</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E5" s="13">
         <v>250</v>
@@ -4278,7 +4266,7 @@
         <v>89</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E6" s="13">
         <v>80</v>
@@ -4754,10 +4742,10 @@
     </row>
     <row r="2" spans="1:14" ht="20" customHeight="1">
       <c r="A2" s="11" t="s">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C2" s="14">
         <v>1180</v>
@@ -4798,10 +4786,10 @@
     </row>
     <row r="3" spans="1:14" ht="20" customHeight="1">
       <c r="A3" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="12" t="s">
         <v>18</v>
-      </c>
-      <c r="B3" s="12" t="s">
-        <v>17</v>
       </c>
       <c r="C3" s="14">
         <v>3400</v>
@@ -4845,7 +4833,7 @@
         <v>19</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C4" s="14">
         <v>1410</v>
@@ -4889,7 +4877,7 @@
         <v>20</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C5" s="14">
         <v>405</v>
@@ -4933,7 +4921,7 @@
         <v>21</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C6" s="14">
         <v>1150</v>
@@ -5377,7 +5365,7 @@
     </row>
     <row r="2" spans="1:5" ht="22" customHeight="1">
       <c r="A2" s="12" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B2" s="15">
         <f>SUMIF(Holdings_Data!$D$2:$D$12, A2, Holdings_Data!$J$2:$J$12)</f>

</xml_diff>